<commit_message>
Adjust Create, 10 testcase for ReadUser
</commit_message>
<xml_diff>
--- a/testdata/TestData.xlsx
+++ b/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Documents\08_Testing\OrangeHRM_Automation_Testing\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388EEAF1-7CE6-4931-9A9A-F4D2F10FD83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6848D6A0-085F-4B29-BD09-19E4E4D438B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="10452" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="verifyCreateUser" sheetId="1" r:id="rId1"/>

</xml_diff>